<commit_message>
Check run 2026-10-28_0909: 4 update(s)
Fix HASiL coverage: Legislation sub-pages are now listed explicitly
(/en/perundangan/ redirects to the Malay site), and crawls follow menu
links, so e-Invoice and e-POS sub-pages are tracked. Re-baselined those
checks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuDWqCNgHsq5MirKxdycYs
</commit_message>
<xml_diff>
--- a/reports/updates-log.xlsx
+++ b/reports/updates-log.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
   <si>
     <t>Run</t>
   </si>
@@ -38,6 +38,90 @@
   </si>
   <si>
     <t>Link</t>
+  </si>
+  <si>
+    <t>2026-10-28_0909</t>
+  </si>
+  <si>
+    <t>Laws of Malaysia (AGC)</t>
+  </si>
+  <si>
+    <t>Principal Act / List of P.U. (A) / Finance Bill (latest legislation feed, tax-relevant only)</t>
+  </si>
+  <si>
+    <t>P.U. (A) 370/2026 – Income Tax (Deduction for Expenditure in relation to Cost of Renovation and Conversion of Office Premise to Residential House) Rules 2026</t>
+  </si>
+  <si>
+    <t>27/10/2026</t>
+  </si>
+  <si>
+    <t>new</t>
+  </si>
+  <si>
+    <t>New further deduction of 10% of the cost of renovating and converting an office premise into a residential house, incurred from 1 January 2026 to 31 December 2027, capped at RM10 million in total; effective from YA 2026. The office premise must have been used for administration/office management for more than 10 years and no longer be in use (shophouses excluded); the conversion plan must be approved by the local authority, the house used solely for habitation and rented out after conversion, and the costs certified by an external auditor. Not available if the same costs were claimed under s.33(1) or as capital allowances under Schedule 2 or 3. Made 24/09/2026.</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://lom.agc.gov.my/ilims/upload/portal/akta/outputp/3793388/P.U.%20(A)%20370_2026.pdf</t>
+  </si>
+  <si>
+    <t>P.U. (A) 371/2026 – Service Tax (Digital Services) (Amendment) Regulations 2026</t>
+  </si>
+  <si>
+    <t>amendment</t>
+  </si>
+  <si>
+    <t>Substitutes regulation 16 (hours for submission of return and payment): returns and payment of service tax or penalty through electronic services can be received at any time except during system maintenance, using Malaysian standard time (UTC+8); where the last day falls on a Federal weekly or public holiday in Malaysia, or a weekly or public holiday in the foreign registered person's country, the deadline is that day. In force 28/10/2026; made 22/10/2026. Also published on MySST on 27/10/2026.</t>
+  </si>
+  <si>
+    <t>Amends the Service Tax (Digital Services) Regulations 2019 [P.U. (A) 269/2019] by substituting regulation 16</t>
+  </si>
+  <si>
+    <t>https://pub-359af8e1f79c472292a7e44ec60f3027.r2.dev/SST%20Regulations/PUA%20371_2026.pdf</t>
+  </si>
+  <si>
+    <t>HASiL (Inland Revenue Board)</t>
+  </si>
+  <si>
+    <t>Home &gt; Kenyataan Media &amp; Pengumuman (Media Statements &amp; Announcements)</t>
+  </si>
+  <si>
+    <t>Operational Guidelines No. 3/2026 – Applications for Tax Clearance Letters (SPC) for Companies, LLPs and Labuan Entities</t>
+  </si>
+  <si>
+    <t>27/10/2026 (announcement); guideline dated 20/10/2026</t>
+  </si>
+  <si>
+    <t>HASiL announced new Operational Guidelines (GPO Bil. 3/2026) on applying for a Tax Clearance Letter for companies, LLPs and Labuan entities, now listed under Legislation &gt; Guidelines. It restates that e-SPC applications through MyTax are mandatory (since 1 January 2024), except Labuan entities and SBMJ, which still submit paper SPC forms. HASiL also relabelled its 'For TCL purpose only' 2026 return forms (C, E, TF, PT) in Download Forms.</t>
+  </si>
+  <si>
+    <t>Covers the same subject as Guideline No. 1/2022 'Application for Tax Clearance Letter for Companies, LLPs and Labuan Entities' (24/05/2022); the new document does not say explicitly that it replaces it</t>
+  </si>
+  <si>
+    <t>https://www.hasil.gov.my/wp-content/uploads/Garis-Panduan-Operasi-Permohonan-SPC-Bagi-Syarikat-Perkongsian-Liabiliti-Terhad-Entiti-Labuan.pdf</t>
+  </si>
+  <si>
+    <t>Chartered Tax Institute of Malaysia</t>
+  </si>
+  <si>
+    <t>eCTIM (titles listed on the public home page; full text needs member sign-in)</t>
+  </si>
+  <si>
+    <t>e-CTIM TECH-IT 41/2026 – Service Tax Policy No. 6/2026 (Amendment No. 1): Improvements to the service tax treatment for electricity transmission and distribution services</t>
+  </si>
+  <si>
+    <t>Not stated (new on CTIM 28/10/2026; RMCD policy dated 26/10/2026)</t>
+  </si>
+  <si>
+    <t>CTIM circulated RMCD's Service Tax Policy No. 6/2026 (Amendment No. 1), which improves the service tax treatment of electricity transmission and distribution services. The full circular is in the CTIM members' area; the policy itself is on MySST's Service Tax Policy page.</t>
+  </si>
+  <si>
+    <t>Amends Service Tax Policy No. 6/2026 (07/10/2026)</t>
+  </si>
+  <si>
+    <t>https://mysst.customs.gov.my/service-tax-policy/</t>
   </si>
 </sst>
 </file>
@@ -76,9 +160,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,7 +505,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -461,8 +548,130 @@
         <v>8</v>
       </c>
     </row>
+    <row r="2" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
+  <hyperlinks>
+    <hyperlink ref="I2" r:id="rId1"/>
+    <hyperlink ref="I3" r:id="rId2"/>
+    <hyperlink ref="I4" r:id="rId3"/>
+    <hyperlink ref="I5" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Check run 2026-10-28_1639: 1 update(s)
Make checks robust to pages that load partially:
- keep a page's previous content when it fails or comes back empty, so
  nothing is reported as removed and nothing is missed afterwards
- drop HASiL's self-redirect parameters from links
- MyTax: wait for the banner slider to load

Re-checks 1656 and 1704 (forms, MyTax, Legislation) only restored items
from the partially loaded visit: no updates.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuDWqCNgHsq5MirKxdycYs
</commit_message>
<xml_diff>
--- a/reports/updates-log.xlsx
+++ b/reports/updates-log.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
   <si>
     <t>Run</t>
   </si>
@@ -122,6 +122,21 @@
   </si>
   <si>
     <t>https://mysst.customs.gov.my/service-tax-policy/</t>
+  </si>
+  <si>
+    <t>2026-10-28_1639</t>
+  </si>
+  <si>
+    <t>Hasilian Research Snapshot (HRS) No. 4/2026 – Perceptions of Individual Taxpayers Among Tax Administrators Toward Adoption of e-Invoice</t>
+  </si>
+  <si>
+    <t>28/10/2026</t>
+  </si>
+  <si>
+    <t>HASiL published a new research snapshot on how tax administrators perceive individual taxpayers' adoption of e-Invoice. It is a research publication, not a ruling or guideline, so it does not change any tax treatment; it may be useful background for e-Invoice discussions.</t>
+  </si>
+  <si>
+    <t>https://www.hasil.gov.my/en/eduzone/penerbitan-cukai/hasilian-research-snapshot-hrs/</t>
   </si>
 </sst>
 </file>
@@ -505,7 +520,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -664,6 +679,35 @@
         <v>36</v>
       </c>
     </row>
+    <row r="6" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <hyperlinks>
@@ -671,6 +715,7 @@
     <hyperlink ref="I3" r:id="rId2"/>
     <hyperlink ref="I4" r:id="rId3"/>
     <hyperlink ref="I5" r:id="rId4"/>
+    <hyperlink ref="I6" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
Check run 2026-10-30_1639: 2 update(s)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuDWqCNgHsq5MirKxdycYs
</commit_message>
<xml_diff>
--- a/reports/updates-log.xlsx
+++ b/reports/updates-log.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
   <si>
     <t>Run</t>
   </si>
@@ -137,6 +137,42 @@
   </si>
   <si>
     <t>https://www.hasil.gov.my/en/eduzone/penerbitan-cukai/hasilian-research-snapshot-hrs/</t>
+  </si>
+  <si>
+    <t>2026-10-30_1639</t>
+  </si>
+  <si>
+    <t>Legislation (everything)</t>
+  </si>
+  <si>
+    <t>Updated online versions of the tax Acts as at 1 January 2026 (ITA 1967, Stamp Act 1949, RPGT Act 1976, LBATA 1990, PITA 1967)</t>
+  </si>
+  <si>
+    <t>30/10/2026 (page last updated 30/10/2026 04:37 PM)</t>
+  </si>
+  <si>
+    <t>replacement</t>
+  </si>
+  <si>
+    <t>HASiL replaced the consolidated online versions of five Acts on its Legislation &gt; Act page with versions as at 1 January 2026: Income Tax Act 1967 (Act 53), Stamp Act 1949 (Act 378), Real Property Gains Tax Act 1976 (Act 169), Labuan Business Activity Tax Act 1990 (Act 445) and Petroleum (Income Tax) Act 1967 (Act 543). The Promotion of Investments Act 1986 stays as at 1 January 2022.</t>
+  </si>
+  <si>
+    <t>Earlier online versions: ITA 1967 (file dated 21/05/2024), Stamp Act 1949 (01/01/2024), RPGT Act 1976 (01/06/2023), LBATA 1990 (01/01/2024); PITA 1967 was already as at 1 January 2026 and was re-uploaded</t>
+  </si>
+  <si>
+    <t>https://www.hasil.gov.my/wp-content/uploads/Income-Tax-Act-1967-online-version-as-at-1-January-2026.pdf</t>
+  </si>
+  <si>
+    <t>Tax case report: MDCOGL v. Director General of Inland Revenue (SCIT, 21/10/2026) – interest income of a non-resident with a PE taxed at 24%, not 15%</t>
+  </si>
+  <si>
+    <t>21/10/2026 (decision); added to HASiL Tax Case page 30/10/2026</t>
+  </si>
+  <si>
+    <t>The Special Commissioners of Income Tax dismissed the appeal of a non-resident company with a permanent establishment in Malaysia, which argued that its Malaysian-sourced interest for YAs 2016–2018 should be taxed at 15% under s.6(1)(b)(i) ITA 1967. The DGIR's position was upheld: the interest was connected to its Malaysian business, so it was taxable at the 24% corporate rate under s.6(1)(a), and the 15% rate only applies where the s.109 withholding mechanism applies. The additional assessments (Form JA) and penalties were confirmed; the taxpayer may appeal within 21 days.</t>
+  </si>
+  <si>
+    <t>https://www.hasil.gov.my/wp-content/uploads/20261021-REVENEWS-MDCOGL.pdf</t>
   </si>
 </sst>
 </file>
@@ -520,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -708,6 +744,64 @@
         <v>41</v>
       </c>
     </row>
+    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <hyperlinks>
@@ -716,6 +810,8 @@
     <hyperlink ref="I4" r:id="rId3"/>
     <hyperlink ref="I5" r:id="rId4"/>
     <hyperlink ref="I6" r:id="rId5"/>
+    <hyperlink ref="I7" r:id="rId6"/>
+    <hyperlink ref="I8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>